<commit_message>
autologin email notification updated
</commit_message>
<xml_diff>
--- a/expedia/templates/Final TimeZoneList (07_12_2018).xlsx
+++ b/expedia/templates/Final TimeZoneList (07_12_2018).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3554fa33ad85cce8/coreOTA/Expedia Templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/darkesthj/Dev/workspace/expedia/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{0791EC40-C077-4755-AA28-0C59CEAEC2E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CC89074-E72D-2647-B399-513CFB9F58CA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597C2166-D856-C846-BDA0-2ADC54CEEB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="1540" windowWidth="28800" windowHeight="15340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -819,10 +819,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>